<commit_message>
fix: map bare 'Marketplace' label into Marketplace group (14 clean groups)
</commit_message>
<xml_diff>
--- a/Yuno_ICP_Bank.xlsx
+++ b/Yuno_ICP_Bank.xlsx
@@ -668,7 +668,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -5706,7 +5706,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -6916,7 +6916,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -9534,7 +9534,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -9952,7 +9952,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -10150,7 +10150,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -10238,7 +10238,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -10392,7 +10392,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -11162,7 +11162,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
@@ -11492,7 +11492,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
@@ -12548,7 +12548,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
@@ -13450,7 +13450,7 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -13582,7 +13582,7 @@
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
@@ -14308,7 +14308,7 @@
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
@@ -14462,7 +14462,7 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -14506,7 +14506,7 @@
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -14814,7 +14814,7 @@
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C667" t="inlineStr">
@@ -15914,7 +15914,7 @@
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
@@ -15936,7 +15936,7 @@
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
@@ -16442,7 +16442,7 @@
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">

</xml_diff>

<commit_message>
fix: fill last missing website (Lemon Cash); 868/868 covered
</commit_message>
<xml_diff>
--- a/Yuno_ICP_Bank.xlsx
+++ b/Yuno_ICP_Bank.xlsx
@@ -14629,7 +14629,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.lemon.me</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>[Argentina] On-ramp routing + card auth uplift</t>

</xml_diff>